<commit_message>
Add deconv annotation table module & outputs
Introduce paper/deconv_annotation_table.py: a new module to build annotation tables from deconvolved FFC maps (per-FFC annotation, b/y matching, ranks matrix, Excel export, and a CLI demo). Add generated outputs and assets (annotation_table_output.xlsx, paper/annotation_table_output*.xlsx, fig1.2.png, partitioned.csv, protein_result.csv). Update pepline code and data (pepline/annotation.py, pepline/deconv_combine.py, pepline/partitioned.csv, pepline/protein_result.csv and result spreadsheets) and adjust paper/graph1.ipynb layout/exec counts. These changes add the annotation generation pipeline and accompanying result files for downstream analysis and reporting.
</commit_message>
<xml_diff>
--- a/pepline/result/mms_annotation.xlsx
+++ b/pepline/result/mms_annotation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevinmbp/Desktop/2D_spec_dict/pepline/result/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B070FDD-1727-EB46-9D69-1D3B19ABA17C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48E6A75F-415D-9F45-B1B9-F375AC94BBC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4860" yWindow="4160" windowWidth="39640" windowHeight="19780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10160" yWindow="30600" windowWidth="29880" windowHeight="16000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="YLE3+" sheetId="2" r:id="rId1"/>
@@ -4788,6 +4788,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="32.83203125" defaultRowHeight="16"/>
+  <cols>
+    <col min="10" max="10" width="40.6640625" customWidth="1"/>
+    <col min="13" max="13" width="43" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Enable visualization, disable saving, clear outputs
Uncomment the visualize_all_paths call in anti_symmetric/anti_symmetric_dp.py and replace the hardcoded desktop save_path with save_path=None so visualizations run without writing to a local file. Update anti_symmetric/comp_anti_symmetric.ipynb execution metadata (clear outputs / reset execution_count) to reduce notebook noise. Remove temporary Office lockfiles (~$...) and update miscellaneous .DS_Store and data/result files tracked in this changeset.
</commit_message>
<xml_diff>
--- a/pepline/result/mms_annotation.xlsx
+++ b/pepline/result/mms_annotation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevinmbp/Desktop/2D_spec_dict/pepline/result/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48E6A75F-415D-9F45-B1B9-F375AC94BBC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB5DA130-1C1F-824D-8425-BBD739575B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10160" yWindow="30600" windowWidth="29880" windowHeight="16000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3400" yWindow="3940" windowWidth="29880" windowHeight="16000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="YLE3+" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1865" uniqueCount="1131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1866" uniqueCount="1132">
   <si>
     <t>N=1000</t>
   </si>
@@ -3419,13 +3419,16 @@
   </si>
   <si>
     <t>(1270.7356, 2842.0915, 4112.8271)</t>
+  </si>
+  <si>
+    <t>s</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -3467,6 +3470,19 @@
       <b/>
       <sz val="12"/>
       <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -3594,7 +3610,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -3617,6 +3633,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4790,7 +4810,10 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="32.83203125" defaultRowHeight="16"/>
   <cols>
     <col min="10" max="10" width="40.6640625" customWidth="1"/>
+    <col min="11" max="11" width="36" customWidth="1"/>
     <col min="13" max="13" width="43" customWidth="1"/>
+    <col min="14" max="14" width="32.83203125" customWidth="1"/>
+    <col min="16" max="16" width="32.83203125" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -4839,7 +4862,7 @@
       <c r="O1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="8" t="s">
         <v>16</v>
       </c>
     </row>
@@ -4856,7 +4879,7 @@
       <c r="O2">
         <v>0</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" s="9" t="s">
         <v>337</v>
       </c>
     </row>
@@ -4873,7 +4896,7 @@
       <c r="O3">
         <v>0</v>
       </c>
-      <c r="P3" t="s">
+      <c r="P3" s="9" t="s">
         <v>339</v>
       </c>
     </row>
@@ -4908,7 +4931,7 @@
       <c r="O4">
         <v>4</v>
       </c>
-      <c r="P4" t="s">
+      <c r="P4" s="9" t="s">
         <v>345</v>
       </c>
     </row>
@@ -4940,7 +4963,7 @@
       <c r="O5">
         <v>3</v>
       </c>
-      <c r="P5" t="s">
+      <c r="P5" s="9" t="s">
         <v>350</v>
       </c>
     </row>
@@ -4972,7 +4995,7 @@
       <c r="O6">
         <v>3</v>
       </c>
-      <c r="P6" t="s">
+      <c r="P6" s="9" t="s">
         <v>355</v>
       </c>
     </row>
@@ -5016,7 +5039,7 @@
       <c r="O7">
         <v>6</v>
       </c>
-      <c r="P7" t="s">
+      <c r="P7" s="9" t="s">
         <v>363</v>
       </c>
     </row>
@@ -5042,7 +5065,7 @@
       <c r="O8">
         <v>2</v>
       </c>
-      <c r="P8" t="s">
+      <c r="P8" s="9" t="s">
         <v>367</v>
       </c>
     </row>
@@ -5086,7 +5109,7 @@
       <c r="O9">
         <v>6</v>
       </c>
-      <c r="P9" t="s">
+      <c r="P9" s="9" t="s">
         <v>375</v>
       </c>
     </row>
@@ -5121,7 +5144,7 @@
       <c r="O10">
         <v>4</v>
       </c>
-      <c r="P10" t="s">
+      <c r="P10" s="9" t="s">
         <v>381</v>
       </c>
     </row>
@@ -5156,7 +5179,7 @@
       <c r="O11">
         <v>4</v>
       </c>
-      <c r="P11" t="s">
+      <c r="P11" s="9" t="s">
         <v>387</v>
       </c>
     </row>
@@ -5200,7 +5223,7 @@
       <c r="O12">
         <v>6</v>
       </c>
-      <c r="P12" t="s">
+      <c r="P12" s="9" t="s">
         <v>395</v>
       </c>
     </row>
@@ -5241,7 +5264,7 @@
       <c r="O13">
         <v>5</v>
       </c>
-      <c r="P13" t="s">
+      <c r="P13" s="9" t="s">
         <v>402</v>
       </c>
     </row>
@@ -5264,7 +5287,7 @@
       <c r="O14">
         <v>1</v>
       </c>
-      <c r="P14" t="s">
+      <c r="P14" s="9" t="s">
         <v>405</v>
       </c>
     </row>
@@ -5290,7 +5313,7 @@
       <c r="O15">
         <v>2</v>
       </c>
-      <c r="P15" t="s">
+      <c r="P15" s="9" t="s">
         <v>409</v>
       </c>
     </row>
@@ -5331,7 +5354,7 @@
       <c r="O16">
         <v>14</v>
       </c>
-      <c r="P16">
+      <c r="P16" s="9">
         <v>14</v>
       </c>
     </row>
@@ -5536,7 +5559,7 @@
       <c r="O33">
         <v>0</v>
       </c>
-      <c r="P33">
+      <c r="P33" s="9">
         <v>0</v>
       </c>
     </row>
@@ -7964,6 +7987,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:R57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="32.83203125" defaultRowHeight="16"/>
+  <cols>
+    <col min="7" max="7" width="54.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:18">
       <c r="A1" s="5" t="s">
@@ -8913,8 +8939,8 @@
       <c r="G38">
         <v>11</v>
       </c>
-      <c r="H38">
-        <v>8</v>
+      <c r="H38" t="s">
+        <v>1131</v>
       </c>
       <c r="J38">
         <v>4</v>

</xml_diff>